<commit_message>
Fix the internal CLB mux mappings for the final bitstream
</commit_message>
<xml_diff>
--- a/bitstream/XACT_comparisons/XC2064_output.xlsx
+++ b/bitstream/XACT_comparisons/XC2064_output.xlsx
@@ -20489,17 +20489,17 @@
           <t>PIP  108G60</t>
         </is>
       </c>
-      <c r="BG25" s="1" t="inlineStr">
+      <c r="BG25" s="2" t="inlineStr">
         <is>
           <t>CLB FF CLK enable</t>
         </is>
       </c>
-      <c r="BH25" s="1" t="inlineStr">
+      <c r="BH25" s="2" t="inlineStr">
         <is>
           <t>CLB FF CLK Invert</t>
         </is>
       </c>
-      <c r="BI25" s="1" t="inlineStr">
+      <c r="BI25" s="2" t="inlineStr">
         <is>
           <t>CLB FF</t>
         </is>
@@ -26715,17 +26715,17 @@
           <t>PIP  148G79</t>
         </is>
       </c>
-      <c r="U33" s="2" t="inlineStr">
+      <c r="U33" s="1" t="inlineStr">
         <is>
           <t>CLB EH CLK enable</t>
         </is>
       </c>
-      <c r="V33" s="2" t="inlineStr">
+      <c r="V33" s="1" t="inlineStr">
         <is>
           <t>CLB EH CLK Invert</t>
         </is>
       </c>
-      <c r="W33" s="2" t="inlineStr">
+      <c r="W33" s="1" t="inlineStr">
         <is>
           <t>CLB EH</t>
         </is>
@@ -26805,12 +26805,12 @@
           <t>PIP  128G79</t>
         </is>
       </c>
-      <c r="AM33" s="2" t="inlineStr">
+      <c r="AM33" s="1" t="inlineStr">
         <is>
           <t>CLB EG CLK enable</t>
         </is>
       </c>
-      <c r="AN33" s="2" t="inlineStr">
+      <c r="AN33" s="1" t="inlineStr">
         <is>
           <t>CLB EG CLK Invert</t>
         </is>
@@ -26905,12 +26905,12 @@
           <t>PIP  108G79</t>
         </is>
       </c>
-      <c r="BG33" s="2" t="inlineStr">
+      <c r="BG33" s="1" t="inlineStr">
         <is>
           <t>CLB EF CLK enable</t>
         </is>
       </c>
-      <c r="BH33" s="2" t="inlineStr">
+      <c r="BH33" s="1" t="inlineStr">
         <is>
           <t>CLB EF CLK Invert</t>
         </is>
@@ -27085,7 +27085,7 @@
           <t>PIP  68G79</t>
         </is>
       </c>
-      <c r="CQ33" s="2" t="inlineStr">
+      <c r="CQ33" s="1" t="inlineStr">
         <is>
           <t>CLB ED CLK enable</t>
         </is>
@@ -27095,7 +27095,7 @@
           <t>CLB ED CLK Invert</t>
         </is>
       </c>
-      <c r="CS33" s="2" t="inlineStr">
+      <c r="CS33" s="1" t="inlineStr">
         <is>
           <t>CLB ED</t>
         </is>
@@ -27185,7 +27185,7 @@
           <t>PIP  48G79</t>
         </is>
       </c>
-      <c r="DK33" s="2" t="inlineStr">
+      <c r="DK33" s="1" t="inlineStr">
         <is>
           <t>CLB EC CLK enable</t>
         </is>
@@ -32494,7 +32494,7 @@
           <t>CLB DF.Y G</t>
         </is>
       </c>
-      <c r="BB40" s="1" t="inlineStr">
+      <c r="BB40" s="2" t="inlineStr">
         <is>
           <t>CLB DF.X G</t>
         </is>
@@ -32589,7 +32589,7 @@
           <t>CLB DE.X G</t>
         </is>
       </c>
-      <c r="BU40" s="1" t="inlineStr">
+      <c r="BU40" s="2" t="inlineStr">
         <is>
           <t>CLB DE.X F/M or Q</t>
         </is>
@@ -32784,7 +32784,7 @@
           <t>CLB DC.X F/M or Q</t>
         </is>
       </c>
-      <c r="DH40" s="2" t="inlineStr">
+      <c r="DH40" s="1" t="inlineStr">
         <is>
           <t>CLB DC Select Latch/FF</t>
         </is>
@@ -33506,7 +33506,7 @@
           <t>CLB DD CLK enable</t>
         </is>
       </c>
-      <c r="CR41" s="1" t="inlineStr">
+      <c r="CR41" s="2" t="inlineStr">
         <is>
           <t>CLB DD CLK Invert</t>
         </is>
@@ -33691,7 +33691,7 @@
           <t>PIP  28G98</t>
         </is>
       </c>
-      <c r="EC41" s="1" t="inlineStr">
+      <c r="EC41" s="2" t="inlineStr">
         <is>
           <t>CLB DB CLK enable</t>
         </is>
@@ -33781,12 +33781,12 @@
           <t>PIP  6G92</t>
         </is>
       </c>
-      <c r="EU41" s="1" t="inlineStr">
+      <c r="EU41" s="2" t="inlineStr">
         <is>
           <t>CLB DA CLK enable</t>
         </is>
       </c>
-      <c r="EV41" s="1" t="inlineStr">
+      <c r="EV41" s="2" t="inlineStr">
         <is>
           <t>CLB DA CLK Invert</t>
         </is>
@@ -38538,7 +38538,7 @@
           <t>CLB CB Logic Table: 1 Bit: 1</t>
         </is>
       </c>
-      <c r="EJ47" s="1" t="inlineStr">
+      <c r="EJ47" s="2" t="inlineStr">
         <is>
           <t>CLB CA Logic Table: 2 Bit: 1</t>
         </is>
@@ -38548,32 +38548,32 @@
           <t>CLB CA Logic Table: 2 Bit: 0</t>
         </is>
       </c>
-      <c r="EL47" s="1" t="inlineStr">
+      <c r="EL47" s="2" t="inlineStr">
         <is>
           <t>CLB CA Logic Table: 2 Bit: 2</t>
         </is>
       </c>
-      <c r="EM47" s="1" t="inlineStr">
+      <c r="EM47" s="2" t="inlineStr">
         <is>
           <t>CLB CA Logic Table: 2 Bit: 3</t>
         </is>
       </c>
-      <c r="EN47" s="1" t="inlineStr">
+      <c r="EN47" s="2" t="inlineStr">
         <is>
           <t>CLB CA Logic Table: 2 Bit: 5</t>
         </is>
       </c>
-      <c r="EO47" s="1" t="inlineStr">
+      <c r="EO47" s="2" t="inlineStr">
         <is>
           <t>CLB CA Logic Table: 2 Bit: 4</t>
         </is>
       </c>
-      <c r="EP47" s="1" t="inlineStr">
+      <c r="EP47" s="2" t="inlineStr">
         <is>
           <t>CLB CA Logic Table: 2 Bit: 6</t>
         </is>
       </c>
-      <c r="EQ47" s="1" t="inlineStr">
+      <c r="EQ47" s="2" t="inlineStr">
         <is>
           <t>CLB CA Logic Table: 2 Bit: 7</t>
         </is>
@@ -38588,32 +38588,32 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="ET47" s="1" t="inlineStr">
+      <c r="ET47" s="2" t="inlineStr">
         <is>
           <t>CLB CA Logic Table: 1 Bit: 7</t>
         </is>
       </c>
-      <c r="EU47" s="1" t="inlineStr">
+      <c r="EU47" s="2" t="inlineStr">
         <is>
           <t>CLB CA Logic Table: 1 Bit: 6</t>
         </is>
       </c>
-      <c r="EV47" s="1" t="inlineStr">
+      <c r="EV47" s="2" t="inlineStr">
         <is>
           <t>CLB CA Logic Table: 1 Bit: 4</t>
         </is>
       </c>
-      <c r="EW47" s="1" t="inlineStr">
+      <c r="EW47" s="2" t="inlineStr">
         <is>
           <t>CLB CA Logic Table: 1 Bit: 5</t>
         </is>
       </c>
-      <c r="EX47" s="1" t="inlineStr">
+      <c r="EX47" s="2" t="inlineStr">
         <is>
           <t>CLB CA Logic Table: 1 Bit: 3</t>
         </is>
       </c>
-      <c r="EY47" s="1" t="inlineStr">
+      <c r="EY47" s="2" t="inlineStr">
         <is>
           <t>CLB CA Logic Table: 1 Bit: 2</t>
         </is>
@@ -38623,7 +38623,7 @@
           <t>CLB CA Logic Table: 1 Bit: 0</t>
         </is>
       </c>
-      <c r="FA47" s="1" t="inlineStr">
+      <c r="FA47" s="2" t="inlineStr">
         <is>
           <t>CLB CA Logic Table: 1 Bit: 1</t>
         </is>
@@ -39340,7 +39340,7 @@
           <t>CLB CB Logic Table: 1 Mux C/D/Q Bit: 1</t>
         </is>
       </c>
-      <c r="EJ48" s="1" t="inlineStr">
+      <c r="EJ48" s="2" t="inlineStr">
         <is>
           <t>CLB CA Logic Table: 2 Mux C/D/Q Bit: 1</t>
         </is>
@@ -39390,12 +39390,12 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="ET48" s="1" t="inlineStr">
+      <c r="ET48" s="2" t="inlineStr">
         <is>
           <t>CLB CA Logic Table: 1 Mux A/B</t>
         </is>
       </c>
-      <c r="EU48" s="1" t="inlineStr">
+      <c r="EU48" s="2" t="inlineStr">
         <is>
           <t>CLB CA Logic Table: 1 Mux B/C</t>
         </is>
@@ -39420,7 +39420,7 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="EZ48" s="1" t="inlineStr">
+      <c r="EZ48" s="2" t="inlineStr">
         <is>
           <t>CLB CA Logic Table: 1 Mux C/D/Q Bit: 0</t>
         </is>
@@ -39842,12 +39842,12 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="CB49" s="1" t="inlineStr">
+      <c r="CB49" s="2" t="inlineStr">
         <is>
           <t>CLB CE Set A/F</t>
         </is>
       </c>
-      <c r="CC49" s="2" t="inlineStr">
+      <c r="CC49" s="1" t="inlineStr">
         <is>
           <t>CLB CE Set-Enable</t>
         </is>
@@ -39937,7 +39937,7 @@
           <t>CLB CD Set A/F</t>
         </is>
       </c>
-      <c r="CU49" s="2" t="inlineStr">
+      <c r="CU49" s="1" t="inlineStr">
         <is>
           <t>CLB CD Set-Enable</t>
         </is>
@@ -40042,12 +40042,12 @@
           <t>CLB CC Set-Enable</t>
         </is>
       </c>
-      <c r="DP49" s="1" t="inlineStr">
+      <c r="DP49" s="2" t="inlineStr">
         <is>
           <t>CLB CC Reset-Enable</t>
         </is>
       </c>
-      <c r="DQ49" s="1" t="inlineStr">
+      <c r="DQ49" s="2" t="inlineStr">
         <is>
           <t>CLB CC Reset D/G</t>
         </is>
@@ -40132,7 +40132,7 @@
           <t>CLB CB Set-Enable</t>
         </is>
       </c>
-      <c r="EH49" s="1" t="inlineStr">
+      <c r="EH49" s="2" t="inlineStr">
         <is>
           <t>CLB CB Reset-Enable</t>
         </is>
@@ -40349,12 +40349,12 @@
           <t>PIP  148G117</t>
         </is>
       </c>
-      <c r="U50" s="1" t="inlineStr">
+      <c r="U50" s="2" t="inlineStr">
         <is>
           <t>CLB CH CLK enable</t>
         </is>
       </c>
-      <c r="V50" s="1" t="inlineStr">
+      <c r="V50" s="2" t="inlineStr">
         <is>
           <t>CLB CH CLK Invert</t>
         </is>
@@ -40439,7 +40439,7 @@
           <t>PIP  128G117</t>
         </is>
       </c>
-      <c r="AM50" s="1" t="inlineStr">
+      <c r="AM50" s="2" t="inlineStr">
         <is>
           <t>CLB CG CLK enable</t>
         </is>
@@ -40449,7 +40449,7 @@
           <t>CLB CG CLK Invert</t>
         </is>
       </c>
-      <c r="AO50" s="1" t="inlineStr">
+      <c r="AO50" s="2" t="inlineStr">
         <is>
           <t>CLB CG</t>
         </is>
@@ -40539,7 +40539,7 @@
           <t>PIP  108G117</t>
         </is>
       </c>
-      <c r="BG50" s="1" t="inlineStr">
+      <c r="BG50" s="2" t="inlineStr">
         <is>
           <t>CLB CF CLK enable</t>
         </is>
@@ -44914,32 +44914,32 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="EB55" s="1" t="inlineStr">
+      <c r="EB55" s="2" t="inlineStr">
         <is>
           <t>CLB BB Logic Table: 1 Bit: 7</t>
         </is>
       </c>
-      <c r="EC55" s="1" t="inlineStr">
+      <c r="EC55" s="2" t="inlineStr">
         <is>
           <t>CLB BB Logic Table: 1 Bit: 6</t>
         </is>
       </c>
-      <c r="ED55" s="1" t="inlineStr">
+      <c r="ED55" s="2" t="inlineStr">
         <is>
           <t>CLB BB Logic Table: 1 Bit: 4</t>
         </is>
       </c>
-      <c r="EE55" s="1" t="inlineStr">
+      <c r="EE55" s="2" t="inlineStr">
         <is>
           <t>CLB BB Logic Table: 1 Bit: 5</t>
         </is>
       </c>
-      <c r="EF55" s="1" t="inlineStr">
+      <c r="EF55" s="2" t="inlineStr">
         <is>
           <t>CLB BB Logic Table: 1 Bit: 3</t>
         </is>
       </c>
-      <c r="EG55" s="1" t="inlineStr">
+      <c r="EG55" s="2" t="inlineStr">
         <is>
           <t>CLB BB Logic Table: 1 Bit: 2</t>
         </is>
@@ -44949,12 +44949,12 @@
           <t>CLB BB Logic Table: 1 Bit: 0</t>
         </is>
       </c>
-      <c r="EI55" s="1" t="inlineStr">
+      <c r="EI55" s="2" t="inlineStr">
         <is>
           <t>CLB BB Logic Table: 1 Bit: 1</t>
         </is>
       </c>
-      <c r="EJ55" s="1" t="inlineStr">
+      <c r="EJ55" s="2" t="inlineStr">
         <is>
           <t>CLB BA Logic Table: 2 Bit: 1</t>
         </is>
@@ -44964,32 +44964,32 @@
           <t>CLB BA Logic Table: 2 Bit: 0</t>
         </is>
       </c>
-      <c r="EL55" s="1" t="inlineStr">
+      <c r="EL55" s="2" t="inlineStr">
         <is>
           <t>CLB BA Logic Table: 2 Bit: 2</t>
         </is>
       </c>
-      <c r="EM55" s="1" t="inlineStr">
+      <c r="EM55" s="2" t="inlineStr">
         <is>
           <t>CLB BA Logic Table: 2 Bit: 3</t>
         </is>
       </c>
-      <c r="EN55" s="1" t="inlineStr">
+      <c r="EN55" s="2" t="inlineStr">
         <is>
           <t>CLB BA Logic Table: 2 Bit: 5</t>
         </is>
       </c>
-      <c r="EO55" s="1" t="inlineStr">
+      <c r="EO55" s="2" t="inlineStr">
         <is>
           <t>CLB BA Logic Table: 2 Bit: 4</t>
         </is>
       </c>
-      <c r="EP55" s="1" t="inlineStr">
+      <c r="EP55" s="2" t="inlineStr">
         <is>
           <t>CLB BA Logic Table: 2 Bit: 6</t>
         </is>
       </c>
-      <c r="EQ55" s="1" t="inlineStr">
+      <c r="EQ55" s="2" t="inlineStr">
         <is>
           <t>CLB BA Logic Table: 2 Bit: 7</t>
         </is>
@@ -45004,32 +45004,32 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="ET55" s="1" t="inlineStr">
+      <c r="ET55" s="2" t="inlineStr">
         <is>
           <t>CLB BA Logic Table: 1 Bit: 7</t>
         </is>
       </c>
-      <c r="EU55" s="1" t="inlineStr">
+      <c r="EU55" s="2" t="inlineStr">
         <is>
           <t>CLB BA Logic Table: 1 Bit: 6</t>
         </is>
       </c>
-      <c r="EV55" s="1" t="inlineStr">
+      <c r="EV55" s="2" t="inlineStr">
         <is>
           <t>CLB BA Logic Table: 1 Bit: 4</t>
         </is>
       </c>
-      <c r="EW55" s="1" t="inlineStr">
+      <c r="EW55" s="2" t="inlineStr">
         <is>
           <t>CLB BA Logic Table: 1 Bit: 5</t>
         </is>
       </c>
-      <c r="EX55" s="1" t="inlineStr">
+      <c r="EX55" s="2" t="inlineStr">
         <is>
           <t>CLB BA Logic Table: 1 Bit: 3</t>
         </is>
       </c>
-      <c r="EY55" s="1" t="inlineStr">
+      <c r="EY55" s="2" t="inlineStr">
         <is>
           <t>CLB BA Logic Table: 1 Bit: 2</t>
         </is>
@@ -45039,7 +45039,7 @@
           <t>CLB BA Logic Table: 1 Bit: 0</t>
         </is>
       </c>
-      <c r="FA55" s="1" t="inlineStr">
+      <c r="FA55" s="2" t="inlineStr">
         <is>
           <t>CLB BA Logic Table: 1 Bit: 1</t>
         </is>
@@ -45716,12 +45716,12 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="EB56" s="1" t="inlineStr">
+      <c r="EB56" s="2" t="inlineStr">
         <is>
           <t>CLB BB Logic Table: 1 Mux A/B</t>
         </is>
       </c>
-      <c r="EC56" s="1" t="inlineStr">
+      <c r="EC56" s="2" t="inlineStr">
         <is>
           <t>CLB BB Logic Table: 1 Mux B/C</t>
         </is>
@@ -45756,7 +45756,7 @@
           <t>CLB BB Logic Table: 1 Mux C/D/Q Bit: 1</t>
         </is>
       </c>
-      <c r="EJ56" s="1" t="inlineStr">
+      <c r="EJ56" s="2" t="inlineStr">
         <is>
           <t>CLB BA Logic Table: 2 Mux C/D/Q Bit: 1</t>
         </is>
@@ -45781,12 +45781,12 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="EO56" s="1" t="inlineStr">
+      <c r="EO56" s="2" t="inlineStr">
         <is>
           <t>CLB BA Logic Table: 2 Mux B/C</t>
         </is>
       </c>
-      <c r="EP56" s="1" t="inlineStr">
+      <c r="EP56" s="2" t="inlineStr">
         <is>
           <t>CLB BA Logic Table: 2 Mux A/B</t>
         </is>
@@ -45806,12 +45806,12 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="ET56" s="1" t="inlineStr">
+      <c r="ET56" s="2" t="inlineStr">
         <is>
           <t>CLB BA Logic Table: 1 Mux A/B</t>
         </is>
       </c>
-      <c r="EU56" s="1" t="inlineStr">
+      <c r="EU56" s="2" t="inlineStr">
         <is>
           <t>CLB BA Logic Table: 1 Mux B/C</t>
         </is>
@@ -45836,7 +45836,7 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="EZ56" s="1" t="inlineStr">
+      <c r="EZ56" s="2" t="inlineStr">
         <is>
           <t>CLB BA Logic Table: 1 Mux C/D/Q Bit: 0</t>
         </is>
@@ -51140,32 +51140,32 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="CP63" s="1" t="inlineStr">
+      <c r="CP63" s="2" t="inlineStr">
         <is>
           <t>CLB AD Logic Table: 1 Bit: 7</t>
         </is>
       </c>
-      <c r="CQ63" s="1" t="inlineStr">
+      <c r="CQ63" s="2" t="inlineStr">
         <is>
           <t>CLB AD Logic Table: 1 Bit: 6</t>
         </is>
       </c>
-      <c r="CR63" s="1" t="inlineStr">
+      <c r="CR63" s="2" t="inlineStr">
         <is>
           <t>CLB AD Logic Table: 1 Bit: 4</t>
         </is>
       </c>
-      <c r="CS63" s="1" t="inlineStr">
+      <c r="CS63" s="2" t="inlineStr">
         <is>
           <t>CLB AD Logic Table: 1 Bit: 5</t>
         </is>
       </c>
-      <c r="CT63" s="1" t="inlineStr">
+      <c r="CT63" s="2" t="inlineStr">
         <is>
           <t>CLB AD Logic Table: 1 Bit: 3</t>
         </is>
       </c>
-      <c r="CU63" s="1" t="inlineStr">
+      <c r="CU63" s="2" t="inlineStr">
         <is>
           <t>CLB AD Logic Table: 1 Bit: 2</t>
         </is>
@@ -51190,7 +51190,7 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="CZ63" s="1" t="inlineStr">
+      <c r="CZ63" s="2" t="inlineStr">
         <is>
           <t>CLB AC Logic Table: 2 Bit: 1</t>
         </is>
@@ -51200,17 +51200,17 @@
           <t>CLB AC Logic Table: 2 Bit: 0</t>
         </is>
       </c>
-      <c r="DB63" s="1" t="inlineStr">
+      <c r="DB63" s="2" t="inlineStr">
         <is>
           <t>CLB AC Logic Table: 2 Bit: 2</t>
         </is>
       </c>
-      <c r="DC63" s="1" t="inlineStr">
+      <c r="DC63" s="2" t="inlineStr">
         <is>
           <t>CLB AC Logic Table: 2 Bit: 3</t>
         </is>
       </c>
-      <c r="DD63" s="1" t="inlineStr">
+      <c r="DD63" s="2" t="inlineStr">
         <is>
           <t>CLB AC Logic Table: 2 Bit: 5</t>
         </is>
@@ -51220,12 +51220,12 @@
           <t>CLB AC Logic Table: 2 Bit: 4</t>
         </is>
       </c>
-      <c r="DF63" s="1" t="inlineStr">
+      <c r="DF63" s="2" t="inlineStr">
         <is>
           <t>CLB AC Logic Table: 2 Bit: 6</t>
         </is>
       </c>
-      <c r="DG63" s="1" t="inlineStr">
+      <c r="DG63" s="2" t="inlineStr">
         <is>
           <t>CLB AC Logic Table: 2 Bit: 7</t>
         </is>
@@ -51240,12 +51240,12 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="DJ63" s="1" t="inlineStr">
+      <c r="DJ63" s="2" t="inlineStr">
         <is>
           <t>CLB AC Logic Table: 1 Bit: 7</t>
         </is>
       </c>
-      <c r="DK63" s="1" t="inlineStr">
+      <c r="DK63" s="2" t="inlineStr">
         <is>
           <t>CLB AC Logic Table: 1 Bit: 6</t>
         </is>
@@ -51255,17 +51255,17 @@
           <t>CLB AC Logic Table: 1 Bit: 4</t>
         </is>
       </c>
-      <c r="DM63" s="1" t="inlineStr">
+      <c r="DM63" s="2" t="inlineStr">
         <is>
           <t>CLB AC Logic Table: 1 Bit: 5</t>
         </is>
       </c>
-      <c r="DN63" s="1" t="inlineStr">
+      <c r="DN63" s="2" t="inlineStr">
         <is>
           <t>CLB AC Logic Table: 1 Bit: 3</t>
         </is>
       </c>
-      <c r="DO63" s="1" t="inlineStr">
+      <c r="DO63" s="2" t="inlineStr">
         <is>
           <t>CLB AC Logic Table: 1 Bit: 2</t>
         </is>
@@ -51275,7 +51275,7 @@
           <t>CLB AC Logic Table: 1 Bit: 0</t>
         </is>
       </c>
-      <c r="DQ63" s="1" t="inlineStr">
+      <c r="DQ63" s="2" t="inlineStr">
         <is>
           <t>CLB AC Logic Table: 1 Bit: 1</t>
         </is>
@@ -51295,7 +51295,7 @@
           <t>CLB AB Logic Table: 2 Bit: 2</t>
         </is>
       </c>
-      <c r="DU63" s="1" t="inlineStr">
+      <c r="DU63" s="2" t="inlineStr">
         <is>
           <t>CLB AB Logic Table: 2 Bit: 3</t>
         </is>
@@ -51315,7 +51315,7 @@
           <t>CLB AB Logic Table: 2 Bit: 6</t>
         </is>
       </c>
-      <c r="DY63" s="1" t="inlineStr">
+      <c r="DY63" s="2" t="inlineStr">
         <is>
           <t>CLB AB Logic Table: 2 Bit: 7</t>
         </is>
@@ -51335,7 +51335,7 @@
           <t>CLB AB Logic Table: 1 Bit: 7</t>
         </is>
       </c>
-      <c r="EC63" s="1" t="inlineStr">
+      <c r="EC63" s="2" t="inlineStr">
         <is>
           <t>CLB AB Logic Table: 1 Bit: 6</t>
         </is>
@@ -51345,12 +51345,12 @@
           <t>CLB AB Logic Table: 1 Bit: 4</t>
         </is>
       </c>
-      <c r="EE63" s="1" t="inlineStr">
+      <c r="EE63" s="2" t="inlineStr">
         <is>
           <t>CLB AB Logic Table: 1 Bit: 5</t>
         </is>
       </c>
-      <c r="EF63" s="1" t="inlineStr">
+      <c r="EF63" s="2" t="inlineStr">
         <is>
           <t>CLB AB Logic Table: 1 Bit: 3</t>
         </is>
@@ -51360,7 +51360,7 @@
           <t>CLB AB Logic Table: 1 Bit: 2</t>
         </is>
       </c>
-      <c r="EH63" s="1" t="inlineStr">
+      <c r="EH63" s="2" t="inlineStr">
         <is>
           <t>CLB AB Logic Table: 1 Bit: 0</t>
         </is>
@@ -51370,7 +51370,7 @@
           <t>CLB AB Logic Table: 1 Bit: 1</t>
         </is>
       </c>
-      <c r="EJ63" s="1" t="inlineStr">
+      <c r="EJ63" s="2" t="inlineStr">
         <is>
           <t>CLB AA Logic Table: 2 Bit: 1</t>
         </is>
@@ -51385,12 +51385,12 @@
           <t>CLB AA Logic Table: 2 Bit: 2</t>
         </is>
       </c>
-      <c r="EM63" s="1" t="inlineStr">
+      <c r="EM63" s="2" t="inlineStr">
         <is>
           <t>CLB AA Logic Table: 2 Bit: 3</t>
         </is>
       </c>
-      <c r="EN63" s="1" t="inlineStr">
+      <c r="EN63" s="2" t="inlineStr">
         <is>
           <t>CLB AA Logic Table: 2 Bit: 5</t>
         </is>
@@ -51405,7 +51405,7 @@
           <t>CLB AA Logic Table: 2 Bit: 6</t>
         </is>
       </c>
-      <c r="EQ63" s="1" t="inlineStr">
+      <c r="EQ63" s="2" t="inlineStr">
         <is>
           <t>CLB AA Logic Table: 2 Bit: 7</t>
         </is>
@@ -51420,7 +51420,7 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="ET63" s="1" t="inlineStr">
+      <c r="ET63" s="2" t="inlineStr">
         <is>
           <t>CLB AA Logic Table: 1 Bit: 7</t>
         </is>
@@ -51435,12 +51435,12 @@
           <t>CLB AA Logic Table: 1 Bit: 4</t>
         </is>
       </c>
-      <c r="EW63" s="1" t="inlineStr">
+      <c r="EW63" s="2" t="inlineStr">
         <is>
           <t>CLB AA Logic Table: 1 Bit: 5</t>
         </is>
       </c>
-      <c r="EX63" s="1" t="inlineStr">
+      <c r="EX63" s="2" t="inlineStr">
         <is>
           <t>CLB AA Logic Table: 1 Bit: 3</t>
         </is>
@@ -51455,7 +51455,7 @@
           <t>CLB AA Logic Table: 1 Bit: 0</t>
         </is>
       </c>
-      <c r="FA63" s="1" t="inlineStr">
+      <c r="FA63" s="2" t="inlineStr">
         <is>
           <t>CLB AA Logic Table: 1 Bit: 1</t>
         </is>
@@ -51942,12 +51942,12 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="CP64" s="1" t="inlineStr">
+      <c r="CP64" s="2" t="inlineStr">
         <is>
           <t>CLB AD Logic Table: 1 Mux A/B</t>
         </is>
       </c>
-      <c r="CQ64" s="1" t="inlineStr">
+      <c r="CQ64" s="2" t="inlineStr">
         <is>
           <t>CLB AD Logic Table: 1 Mux B/C</t>
         </is>
@@ -51972,7 +51972,7 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="CV64" s="1" t="inlineStr">
+      <c r="CV64" s="2" t="inlineStr">
         <is>
           <t>CLB AD Logic Table: 1 Mux C/D/Q Bit: 0</t>
         </is>
@@ -51992,7 +51992,7 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="CZ64" s="1" t="inlineStr">
+      <c r="CZ64" s="2" t="inlineStr">
         <is>
           <t>CLB AC Logic Table: 2 Mux C/D/Q Bit: 1</t>
         </is>
@@ -52017,12 +52017,12 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="DE64" s="1" t="inlineStr">
+      <c r="DE64" s="2" t="inlineStr">
         <is>
           <t>CLB AC Logic Table: 2 Mux B/C</t>
         </is>
       </c>
-      <c r="DF64" s="1" t="inlineStr">
+      <c r="DF64" s="2" t="inlineStr">
         <is>
           <t>CLB AC Logic Table: 2 Mux A/B</t>
         </is>
@@ -52042,7 +52042,7 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="DJ64" s="1" t="inlineStr">
+      <c r="DJ64" s="2" t="inlineStr">
         <is>
           <t>CLB AC Logic Table: 1 Mux A/B</t>
         </is>
@@ -52077,12 +52077,12 @@
           <t>CLB AC Logic Table: 1 Mux C/D/Q Bit: 0</t>
         </is>
       </c>
-      <c r="DQ64" s="1" t="inlineStr">
+      <c r="DQ64" s="2" t="inlineStr">
         <is>
           <t>CLB AC Logic Table: 1 Mux C/D/Q Bit: 1</t>
         </is>
       </c>
-      <c r="DR64" s="1" t="inlineStr">
+      <c r="DR64" s="2" t="inlineStr">
         <is>
           <t>CLB AB Logic Table: 2 Mux C/D/Q Bit: 1</t>
         </is>
@@ -52107,12 +52107,12 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="DW64" s="1" t="inlineStr">
+      <c r="DW64" s="2" t="inlineStr">
         <is>
           <t>CLB AB Logic Table: 2 Mux B/C</t>
         </is>
       </c>
-      <c r="DX64" s="1" t="inlineStr">
+      <c r="DX64" s="2" t="inlineStr">
         <is>
           <t>CLB AB Logic Table: 2 Mux A/B</t>
         </is>
@@ -52132,12 +52132,12 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="EB64" s="1" t="inlineStr">
+      <c r="EB64" s="2" t="inlineStr">
         <is>
           <t>CLB AB Logic Table: 1 Mux A/B</t>
         </is>
       </c>
-      <c r="EC64" s="1" t="inlineStr">
+      <c r="EC64" s="2" t="inlineStr">
         <is>
           <t>CLB AB Logic Table: 1 Mux B/C</t>
         </is>
@@ -52162,7 +52162,7 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="EH64" s="1" t="inlineStr">
+      <c r="EH64" s="2" t="inlineStr">
         <is>
           <t>CLB AB Logic Table: 1 Mux C/D/Q Bit: 0</t>
         </is>
@@ -52177,7 +52177,7 @@
           <t>CLB AA Logic Table: 2 Mux C/D/Q Bit: 1</t>
         </is>
       </c>
-      <c r="EK64" s="1" t="inlineStr">
+      <c r="EK64" s="2" t="inlineStr">
         <is>
           <t>CLB AA Logic Table: 2 Mux C/D/Q Bit: 0</t>
         </is>
@@ -52202,7 +52202,7 @@
           <t>CLB AA Logic Table: 2 Mux B/C</t>
         </is>
       </c>
-      <c r="EP64" s="1" t="inlineStr">
+      <c r="EP64" s="2" t="inlineStr">
         <is>
           <t>CLB AA Logic Table: 2 Mux A/B</t>
         </is>
@@ -52252,7 +52252,7 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="EZ64" s="1" t="inlineStr">
+      <c r="EZ64" s="2" t="inlineStr">
         <is>
           <t>CLB AA Logic Table: 1 Mux C/D/Q Bit: 0</t>
         </is>

</xml_diff>